<commit_message>
general update for dissertation stuff
</commit_message>
<xml_diff>
--- a/Hysteresis/Experiments-Summer2022/Exp2022_Hydrographs.xlsx
+++ b/Hysteresis/Experiments-Summer2022/Exp2022_Hydrographs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\GitHub\La_Jara\Hysteresis\Experiments-Summer2022\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\La_Jara\Hysteresis\Experiments-Summer2022\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6FD96B1-A77E-4531-86A6-7830A4DB50D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7F068A4-8932-44FD-A495-66966FB726CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{055D4222-03BB-4B33-97D6-42AEC377BEC2}"/>
   </bookViews>
@@ -795,6 +795,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="37644799"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
@@ -838,6 +839,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -845,7 +847,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1534,6 +1535,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1541,7 +1543,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2247,6 +2248,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2254,7 +2256,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2972,6 +2973,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2979,7 +2981,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3675,6 +3676,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3682,7 +3684,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4384,6 +4385,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4391,7 +4393,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5122,6 +5123,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5129,7 +5131,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5884,6 +5885,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5891,7 +5893,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6610,6 +6611,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6617,7 +6619,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7371,6 +7372,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7378,7 +7380,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8096,6 +8097,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8103,7 +8105,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8804,6 +8805,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8811,7 +8813,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9524,6 +9525,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9531,7 +9533,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10208,6 +10209,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10215,7 +10217,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -18549,9 +18550,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -18589,7 +18590,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -18695,7 +18696,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -18837,7 +18838,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -18846,13 +18847,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A894D1A4-D2B6-4A55-85C6-2598F77D3B77}">
   <dimension ref="A1:AO18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="7" max="11" width="9.140625" style="1"/>
-    <col min="13" max="17" width="9.140625" style="1"/>
+    <col min="7" max="11" width="9.109375" style="1"/>
+    <col min="13" max="17" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -18903,7 +18904,7 @@
       <c r="AN1" s="3"/>
       <c r="AO1" s="3"/>
     </row>
-    <row r="2" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -19010,7 +19011,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -19117,7 +19118,7 @@
         <v>3.0339999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -19224,7 +19225,7 @@
         <v>3.0539999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -19331,7 +19332,7 @@
         <v>2.4729999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -19438,7 +19439,7 @@
         <v>2.6160000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -19545,7 +19546,7 @@
         <v>3.1349999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -19652,7 +19653,7 @@
         <v>2.9359999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -19759,7 +19760,7 @@
         <v>2.9329999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -19866,7 +19867,7 @@
         <v>2.6339999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -19973,7 +19974,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="12" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -20080,7 +20081,7 @@
         <v>2.97</v>
       </c>
     </row>
-    <row r="13" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -20187,7 +20188,7 @@
         <v>2.4969999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -20264,7 +20265,7 @@
         <v>2.883</v>
       </c>
     </row>
-    <row r="15" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -20326,7 +20327,7 @@
         <v>2.84</v>
       </c>
     </row>
-    <row r="16" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:41" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -20358,7 +20359,7 @@
         <v>2.7410000000000001</v>
       </c>
     </row>
-    <row r="17" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G17" s="1">
         <v>15</v>
       </c>
@@ -20375,7 +20376,7 @@
         <v>2.7519999999999998</v>
       </c>
     </row>
-    <row r="18" spans="7:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G18" s="1">
         <v>16</v>
       </c>

</xml_diff>